<commit_message>
Replacing old version of Part 1 Excel
</commit_message>
<xml_diff>
--- a/Q3 - MS Project.xlsx
+++ b/Q3 - MS Project.xlsx
@@ -10,7 +10,7 @@
     <sheet sheetId="1" r:id="rId1" name="Task_Table1"/>
   </sheets>
   <definedNames>
-    <definedName name="Task_Table1">'Task_Table1'!$A$1:$H$1</definedName>
+    <definedName name="Task_Table1">'Task_Table1'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
@@ -343,7 +343,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row outlineLevel="0" r="1">
@@ -364,27 +364,17 @@
       </c>
       <c r="D1" s="0" t="inlineStr">
         <is>
-          <t>Scheduled_Start</t>
+          <t>Predecessors</t>
         </is>
       </c>
       <c r="E1" s="0" t="inlineStr">
         <is>
+          <t>Start_Date</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
           <t>Finish_Date</t>
-        </is>
-      </c>
-      <c r="F1" s="0" t="inlineStr">
-        <is>
-          <t>Predecessors</t>
-        </is>
-      </c>
-      <c r="G1" s="0" t="inlineStr">
-        <is>
-          <t>Resource_Names</t>
-        </is>
-      </c>
-      <c r="H1" s="0" t="inlineStr">
-        <is>
-          <t>Cost</t>
         </is>
       </c>
     </row>
@@ -401,22 +391,17 @@
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>225 days</t>
-        </is>
-      </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t>Thu 1/1/26</t>
+          <t>195 days</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t>November 12, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="H2" s="0" t="inlineStr">
-        <is>
-          <t>1625920</t>
+          <t>January 1, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>September 30, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -436,19 +421,14 @@
           <t>30 days</t>
         </is>
       </c>
-      <c r="D3" s="0" t="inlineStr">
-        <is>
-          <t>Thu 1/1/26</t>
-        </is>
-      </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
+          <t>January 1, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
           <t>February 11, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H3" s="0" t="inlineStr">
-        <is>
-          <t>132000</t>
         </is>
       </c>
     </row>
@@ -468,19 +448,14 @@
           <t>15 days</t>
         </is>
       </c>
-      <c r="D4" s="0" t="inlineStr">
-        <is>
-          <t>Thu 1/1/26</t>
-        </is>
-      </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
+          <t>January 1, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
           <t>January 22, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="H4" s="0" t="inlineStr">
-        <is>
-          <t>66000</t>
         </is>
       </c>
     </row>
@@ -500,24 +475,14 @@
           <t>7 days</t>
         </is>
       </c>
-      <c r="D5" s="0" t="inlineStr">
-        <is>
-          <t>Tue 10/7/25</t>
-        </is>
-      </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
+          <t>January 1, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
           <t>January 9, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="G5" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="H5" s="0" t="inlineStr">
-        <is>
-          <t>30800</t>
         </is>
       </c>
     </row>
@@ -539,27 +504,17 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>Mon 1/12/26</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
+          <t>January 12, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
           <t>January 21, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F6" s="0" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G6" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="H6" s="0" t="inlineStr">
-        <is>
-          <t>35200</t>
         </is>
       </c>
     </row>
@@ -581,7 +536,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>Wed 1/21/26</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -591,12 +546,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H7" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>January 22, 2026 8:00 AM</t>
         </is>
       </c>
     </row>
@@ -616,19 +566,14 @@
           <t>15 days</t>
         </is>
       </c>
-      <c r="D8" s="0" t="inlineStr">
-        <is>
-          <t>Thu 1/22/26</t>
-        </is>
-      </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
+          <t>January 22, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
           <t>February 11, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H8" s="0" t="inlineStr">
-        <is>
-          <t>66000</t>
         </is>
       </c>
     </row>
@@ -650,27 +595,17 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>Thu 1/22/26</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
+          <t>January 22, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
           <t>February 2, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F9" s="0" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G9" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="H9" s="0" t="inlineStr">
-        <is>
-          <t>35200</t>
         </is>
       </c>
     </row>
@@ -692,27 +627,17 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>Tue 2/3/26</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
+          <t>February 3, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
           <t>February 11, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F10" s="0" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="G10" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="H10" s="0" t="inlineStr">
-        <is>
-          <t>30800</t>
         </is>
       </c>
     </row>
@@ -734,22 +659,17 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>Thu 2/12/26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
+          <t>February 12, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
           <t>April 23, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="F11" s="0" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H11" s="0" t="inlineStr">
-        <is>
-          <t>343200</t>
         </is>
       </c>
     </row>
@@ -769,19 +689,14 @@
           <t>25 days</t>
         </is>
       </c>
-      <c r="D12" s="0" t="inlineStr">
-        <is>
-          <t>Thu 2/12/26</t>
-        </is>
-      </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
+          <t>February 12, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
           <t>March 18, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H12" s="0" t="inlineStr">
-        <is>
-          <t>190000</t>
         </is>
       </c>
     </row>
@@ -803,27 +718,17 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>Thu 2/12/26</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
+          <t>February 12, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
           <t>February 27, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="G13" s="0" t="inlineStr">
-        <is>
-          <t>UI/UX Designer ,Project Manager</t>
-        </is>
-      </c>
-      <c r="H13" s="0" t="inlineStr">
-        <is>
-          <t>91200</t>
         </is>
       </c>
     </row>
@@ -845,27 +750,17 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>Mon 3/2/26</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
+          <t>March 2, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
           <t>March 18, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F14" s="0" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G14" s="0" t="inlineStr">
-        <is>
-          <t>UI/UX Designer ,Project Manager</t>
-        </is>
-      </c>
-      <c r="H14" s="0" t="inlineStr">
-        <is>
-          <t>98800</t>
         </is>
       </c>
     </row>
@@ -885,19 +780,14 @@
           <t>25 days</t>
         </is>
       </c>
-      <c r="D15" s="0" t="inlineStr">
-        <is>
-          <t>Thu 3/19/26</t>
-        </is>
-      </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
+          <t>March 19, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
           <t>April 23, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="H15" s="0" t="inlineStr">
-        <is>
-          <t>153200</t>
         </is>
       </c>
     </row>
@@ -919,27 +809,17 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Thu 3/19/26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
+          <t>March 19, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
           <t>April 3, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F16" s="0" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="G16" s="0" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="H16" s="0" t="inlineStr">
-        <is>
-          <t>46080</t>
         </is>
       </c>
     </row>
@@ -961,27 +841,17 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>Mon 4/6/26</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
+          <t>April 6, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
           <t>April 22, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F17" s="0" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="G17" s="0" t="inlineStr">
-        <is>
-          <t>Software Engineer,Project Manager</t>
-        </is>
-      </c>
-      <c r="H17" s="0" t="inlineStr">
-        <is>
-          <t>107120</t>
         </is>
       </c>
     </row>
@@ -1003,7 +873,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>Wed 4/22/26</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -1013,12 +883,7 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H18" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>April 23, 2026 8:00 AM</t>
         </is>
       </c>
     </row>
@@ -1035,27 +900,22 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>90 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>Thu 4/23/26</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>August 27, 2026 8:00 AM</t>
+          <t>April 23, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="H19" s="0" t="inlineStr">
-        <is>
-          <t>659200</t>
+          <t>July 15, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1072,22 +932,17 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>30 days</t>
-        </is>
-      </c>
-      <c r="D20" s="0" t="inlineStr">
-        <is>
-          <t>Thu 4/23/26</t>
+          <t>20 days</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>June 3, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H20" s="0" t="inlineStr">
-        <is>
-          <t>105600</t>
+          <t>April 23, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>May 20, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1109,27 +964,17 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>Thu 4/23/26</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
+          <t>April 23, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
           <t>May 6, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="F21" s="0" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G21" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer</t>
-        </is>
-      </c>
-      <c r="H21" s="0" t="inlineStr">
-        <is>
-          <t>33600</t>
         </is>
       </c>
     </row>
@@ -1151,27 +996,17 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>Thu 5/7/26</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>May 20, 2026 5:00 PM</t>
+          <t>April 23, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="G22" s="0" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="H22" s="0" t="inlineStr">
-        <is>
-          <t>38400.000000000007</t>
+          <t>May 6, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1193,27 +1028,17 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>Thu 5/21/26</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>June 3, 2026 5:00 PM</t>
+          <t>May 7, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="G23" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer</t>
-        </is>
-      </c>
-      <c r="H23" s="0" t="inlineStr">
-        <is>
-          <t>33600</t>
+          <t>May 20, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1230,22 +1055,17 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>30 days</t>
-        </is>
-      </c>
-      <c r="D24" s="0" t="inlineStr">
-        <is>
-          <t>Thu 6/4/26</t>
+          <t>20 days</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>July 15, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H24" s="0" t="inlineStr">
-        <is>
-          <t>343200</t>
+          <t>May 21, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>June 17, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1267,27 +1087,17 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>Thu 6/4/26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>June 17, 2026 5:00 PM</t>
+          <t>May 21, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="G25" s="0" t="inlineStr">
-        <is>
-          <t>Software Engineer,UI/UX Designer ,Project Manager</t>
-        </is>
-      </c>
-      <c r="H25" s="0" t="inlineStr">
-        <is>
-          <t>114400</t>
+          <t>June 3, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1309,27 +1119,17 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>Thu 6/18/26</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>July 1, 2026 5:00 PM</t>
+          <t>June 4, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="G26" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,Software Engineer,UI/UX Designer</t>
-        </is>
-      </c>
-      <c r="H26" s="0" t="inlineStr">
-        <is>
-          <t>114400</t>
+          <t>June 17, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1351,27 +1151,17 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>Thu 7/2/26</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>July 15, 2026 5:00 PM</t>
+          <t>June 4, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="G27" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,Software Engineer,UI/UX Designer</t>
-        </is>
-      </c>
-      <c r="H27" s="0" t="inlineStr">
-        <is>
-          <t>114400</t>
+          <t>June 17, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1388,22 +1178,17 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>30 days</t>
-        </is>
-      </c>
-      <c r="D28" s="0" t="inlineStr">
-        <is>
-          <t>Thu 7/16/26</t>
+          <t>20 days</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>August 27, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="H28" s="0" t="inlineStr">
-        <is>
-          <t>210400</t>
+          <t>June 18, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>July 15, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1425,27 +1210,17 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>Thu 7/16/26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>July 29, 2026 5:00 PM</t>
+          <t>June 18, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="G29" s="0" t="inlineStr">
-        <is>
-          <t>Software Engineer,UI/UX Designer</t>
-        </is>
-      </c>
-      <c r="H29" s="0" t="inlineStr">
-        <is>
-          <t>70400</t>
+          <t>July 1, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1467,27 +1242,17 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>Thu 7/30/26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>August 12, 2026 5:00 PM</t>
+          <t>July 2, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="G30" s="0" t="inlineStr">
-        <is>
-          <t>QA Tester,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H30" s="0" t="inlineStr">
-        <is>
-          <t>67200</t>
+          <t>July 15, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1509,27 +1274,17 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>Thu 8/13/26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>August 26, 2026 5:00 PM</t>
+          <t>July 2, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="G31" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,QA Tester</t>
-        </is>
-      </c>
-      <c r="H31" s="0" t="inlineStr">
-        <is>
-          <t>72800</t>
+          <t>July 15, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1551,22 +1306,17 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>Wed 8/26/26</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>August 27, 2026 8:00 AM</t>
+          <t>July 15, 2026 5:00 PM</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="H32" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>July 15, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1588,22 +1338,17 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>Thu 8/27/26</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>October 8, 2026 8:00 AM</t>
+          <t>July 16, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="H33" s="0" t="inlineStr">
-        <is>
-          <t>268160</t>
+          <t>August 26, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1623,19 +1368,14 @@
           <t>15 days</t>
         </is>
       </c>
-      <c r="D34" s="0" t="inlineStr">
-        <is>
-          <t>Thu 8/27/26</t>
-        </is>
-      </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>September 16, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t>159520</t>
+          <t>July 16, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>August 5, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1657,27 +1397,17 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>Thu 8/27/26</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>September 7, 2026 5:00 PM</t>
+          <t>July 16, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="G35" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,QA Tester,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H35" s="0" t="inlineStr">
-        <is>
-          <t>88960</t>
+          <t>July 27, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1699,27 +1429,17 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>Tue 9/8/26</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>September 16, 2026 5:00 PM</t>
+          <t>July 28, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="G36" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer,QA Tester,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H36" s="0" t="inlineStr">
-        <is>
-          <t>70560</t>
+          <t>August 5, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1739,19 +1459,14 @@
           <t>15 days</t>
         </is>
       </c>
-      <c r="D37" s="0" t="inlineStr">
-        <is>
-          <t>Thu 9/17/26</t>
-        </is>
-      </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>October 8, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="H37" s="0" t="inlineStr">
-        <is>
-          <t>108640</t>
+          <t>August 6, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>August 26, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1773,27 +1488,17 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>Thu 9/17/26</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>September 28, 2026 5:00 PM</t>
+          <t>August 6, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="G38" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,QA Tester</t>
-        </is>
-      </c>
-      <c r="H38" s="0" t="inlineStr">
-        <is>
-          <t>58240</t>
+          <t>August 17, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1815,27 +1520,17 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>Tue 9/29/26</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>October 7, 2026 5:00 PM</t>
+          <t>August 18, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="G39" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H39" s="0" t="inlineStr">
-        <is>
-          <t>50400</t>
+          <t>August 26, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1552,17 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>Wed 10/7/26</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>October 8, 2026 8:00 AM</t>
+          <t>August 26, 2026 5:00 PM</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="H40" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>August 26, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1894,22 +1584,17 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>Thu 10/8/26</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>October 29, 2026 8:00 AM</t>
+          <t>August 27, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="H41" s="0" t="inlineStr">
-        <is>
-          <t>189360</t>
+          <t>September 16, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1929,19 +1614,14 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="D42" s="0" t="inlineStr">
-        <is>
-          <t>Thu 10/8/26</t>
-        </is>
-      </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>October 14, 2026 5:00 PM</t>
-        </is>
-      </c>
-      <c r="H42" s="0" t="inlineStr">
-        <is>
-          <t>73360</t>
+          <t>August 27, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>September 2, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -1963,27 +1643,17 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>Thu 10/8/26</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>October 12, 2026 5:00 PM</t>
+          <t>August 27, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="G43" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer,UI/UX Designer ,Project Manager,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H43" s="0" t="inlineStr">
-        <is>
-          <t>44400</t>
+          <t>August 31, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2005,27 +1675,17 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Tue 10/13/26</t>
+          <t>41</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>October 14, 2026 5:00 PM</t>
+          <t>September 1, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="G44" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer,Project Manager,QA Tester,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H44" s="0" t="inlineStr">
-        <is>
-          <t>28960</t>
+          <t>September 2, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2045,19 +1705,14 @@
           <t>10 days</t>
         </is>
       </c>
-      <c r="D45" s="0" t="inlineStr">
-        <is>
-          <t>Thu 10/15/26</t>
-        </is>
-      </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>October 29, 2026 8:00 AM</t>
-        </is>
-      </c>
-      <c r="H45" s="0" t="inlineStr">
-        <is>
-          <t>116000</t>
+          <t>September 3, 2026 8:00 AM</t>
+        </is>
+      </c>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t>September 16, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2079,27 +1734,17 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Thu 10/15/26</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>October 21, 2026 5:00 PM</t>
+          <t>September 3, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="G46" s="0" t="inlineStr">
-        <is>
-          <t>DevOps Engineer,Project Manager,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H46" s="0" t="inlineStr">
-        <is>
-          <t>58000</t>
+          <t>September 9, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2121,27 +1766,17 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Thu 10/22/26</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>October 28, 2026 5:00 PM</t>
+          <t>September 10, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="G47" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,DevOps Engineer,Software Engineer</t>
-        </is>
-      </c>
-      <c r="H47" s="0" t="inlineStr">
-        <is>
-          <t>58000</t>
+          <t>September 16, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2163,22 +1798,17 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>Wed 10/28/26</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>October 29, 2026 8:00 AM</t>
+          <t>September 16, 2026 5:00 PM</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="H48" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>September 16, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2200,22 +1830,17 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Thu 10/29/26</t>
+          <t>39</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>November 12, 2026 8:00 AM</t>
+          <t>September 17, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="H49" s="0" t="inlineStr">
-        <is>
-          <t>34000</t>
+          <t>September 30, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2237,22 +1862,17 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Thu 10/29/26</t>
+          <t>46</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>November 4, 2026 5:00 PM</t>
+          <t>September 17, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="H50" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>September 23, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2274,27 +1894,17 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>Thu 11/5/26</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>November 9, 2026 5:00 PM</t>
+          <t>September 24, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="G51" s="0" t="inlineStr">
-        <is>
-          <t>Finance/Admin Officer,Project Manager</t>
-        </is>
-      </c>
-      <c r="H51" s="0" t="inlineStr">
-        <is>
-          <t>20400</t>
+          <t>September 28, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2316,27 +1926,17 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Tue 11/10/26</t>
+          <t>49</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>November 11, 2026 5:00 PM</t>
+          <t>September 29, 2026 8:00 AM</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="G52" s="0" t="inlineStr">
-        <is>
-          <t>Project Manager,Finance/Admin Officer</t>
-        </is>
-      </c>
-      <c r="H52" s="0" t="inlineStr">
-        <is>
-          <t>13600</t>
+          <t>September 30, 2026 5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2358,22 +1958,17 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>Wed 11/11/26</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>November 12, 2026 8:00 AM</t>
+          <t>September 30, 2026 5:00 PM</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="H53" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>September 30, 2026 5:00 PM</t>
         </is>
       </c>
     </row>

</xml_diff>